<commit_message>
Backfill vacancy counts for 3 and 4 October 2026
No report ran on 3 or 4 October, because the Worker's GH_TOKEN had been
regenerated on GitHub without the new value being stored in the Worker,
so the analytics series had no rows for those days.

The 4 October row is a real reading: the board totals were scraped with
scrapers.fetch_all() at 23:19 Kyiv time on that day, with no errors
(DOU 226, Djinni 61).

The 3 October row is an estimate, not a measurement. The boards only
report their current totals, so that day cannot be read after the fact.
It is the mean of the 2 and 4 October readings (DOU 234, Djinni 65,
rounded half up), chosen by the owner over leaving a gap. The CSV has no
way to flag an estimated row, so this commit is the record of it.

The workbook was regenerated from the CSV with analytics.build_workbook().

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/vacancy-analytics.xlsx
+++ b/reports/vacancy-analytics.xlsx
@@ -168,12 +168,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2:$A$24</f>
+              <f>'Counts'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$B$2:$B$24</f>
+              <f>'Counts'!$B$2:$B$26</f>
             </numRef>
           </val>
         </ser>
@@ -200,12 +200,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2:$A$24</f>
+              <f>'Counts'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$C$2:$C$24</f>
+              <f>'Counts'!$C$2:$C$26</f>
             </numRef>
           </val>
         </ser>
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -907,6 +907,32 @@
       </c>
       <c r="C24" t="n">
         <v>68</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>234</v>
+      </c>
+      <c r="C25" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>226</v>
+      </c>
+      <c r="C26" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backfill vacancy counts for 3 and 4 October 2026 (#151)
No report ran on 3 or 4 October, because the Worker's GH_TOKEN had been
regenerated on GitHub without the new value being stored in the Worker,
so the analytics series had no rows for those days.

The 4 October row is a real reading: the board totals were scraped with
scrapers.fetch_all() at 23:19 Kyiv time on that day, with no errors
(DOU 226, Djinni 61).

The 3 October row is an estimate, not a measurement. The boards only
report their current totals, so that day cannot be read after the fact.
It is the mean of the 2 and 4 October readings (DOU 234, Djinni 65,
rounded half up), chosen by the owner over leaving a gap. The CSV has no
way to flag an estimated row, so this commit is the record of it.

The workbook was regenerated from the CSV with analytics.build_workbook().

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/vacancy-analytics.xlsx
+++ b/reports/vacancy-analytics.xlsx
@@ -168,12 +168,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2:$A$24</f>
+              <f>'Counts'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$B$2:$B$24</f>
+              <f>'Counts'!$B$2:$B$26</f>
             </numRef>
           </val>
         </ser>
@@ -200,12 +200,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Counts'!$A$2:$A$24</f>
+              <f>'Counts'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Counts'!$C$2:$C$24</f>
+              <f>'Counts'!$C$2:$C$26</f>
             </numRef>
           </val>
         </ser>
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -907,6 +907,32 @@
       </c>
       <c r="C24" t="n">
         <v>68</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>234</v>
+      </c>
+      <c r="C25" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>226</v>
+      </c>
+      <c r="C26" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>